<commit_message>
feat(moves): add human decision controls
</commit_message>
<xml_diff>
--- a/docs/planning/ABARVA_PILOT_READINESS_PLAN.xlsx
+++ b/docs/planning/ABARVA_PILOT_READINESS_PLAN.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Radae33b0ee4f4611"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R8802abbdeca6425a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan" sheetId="3" r:id="R922cf2536a504dcd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Queue" sheetId="4" r:id="Rf6d85ccb547143c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance" sheetId="5" r:id="R35f78e8629d0406a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pricing" sheetId="6" r:id="R783204f43a344bea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost Model" sheetId="7" r:id="R8ddd5e1ea0164c88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BC - PHS" sheetId="8" r:id="R2b7350b4cd2c44e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BC - Surekha" sheetId="9" r:id="R5e274a997fb1459b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BC - Delta" sheetId="10" r:id="Rd0b0fcaa3e544037"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Pack" sheetId="11" r:id="Rdfbfb49120284963"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Redline Brief" sheetId="12" r:id="R3293ef2d4ddc4220"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="13" r:id="Rcb3731a14a2e4bfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R2fa155bca9184c28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Ra751f8589b5f4dc3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan" sheetId="3" r:id="R2ba836e4f62f4681"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Queue" sheetId="4" r:id="Rcd96f3fadf154750"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance" sheetId="5" r:id="Re2f9f7c512b6412f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pricing" sheetId="6" r:id="R3a9496baee504c9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost Model" sheetId="7" r:id="R003202e93e884977"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BC - PHS" sheetId="8" r:id="Rb50ecf56ccf74679"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BC - Surekha" sheetId="9" r:id="R3fda1d3bdfe44112"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BC - Delta" sheetId="10" r:id="R9a8442473fe54da2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Pack" sheetId="11" r:id="R1a189b3f5ce14818"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Redline Brief" sheetId="12" r:id="R3152d3b9b0544921"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="13" r:id="R1437e39d35404035"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4599,7 +4599,7 @@
       </x:c>
       <x:c r="C8" s="7" t="n">
         <x:f>COUNTIF(Plan!L5:L333,"In progress")</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G8" s="6" t="inlineStr">
         <x:is>
@@ -4663,7 +4663,7 @@
       </x:c>
       <x:c r="C10" s="7" t="n">
         <x:f>COUNTIF(Plan!L5:L333,"Not started")</x:f>
-        <x:v>328</x:v>
+        <x:v>325</x:v>
       </x:c>
       <x:c r="G10" s="6" t="inlineStr">
         <x:is>
@@ -5090,7 +5090,7 @@
       </x:c>
       <x:c r="J20" s="9" t="n">
         <x:f>COUNTIFS(Plan!B5:B333,"AI Liability Defense",Plan!L5:L333,"In progress")</x:f>
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K20" s="10" t="n">
         <x:f>IFERROR(I20/H20,0)</x:f>
@@ -7691,15 +7691,11 @@
           <x:t xml:space="preserve">Anytime</x:t>
         </x:is>
       </x:c>
-      <x:c r="L25" s="44" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M25" s="18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
+      <x:c r="L25" s="44" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="M25" s="18" t="str">
+        <x:v>codex/moves-ai-liability-retrofit: adds 20-char human gate rationale and shared AI decision evidence packet to Moves phase-gate approval paths.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -7758,15 +7754,11 @@
           <x:t xml:space="preserve">Pre-Resign</x:t>
         </x:is>
       </x:c>
-      <x:c r="L26" s="44" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M26" s="18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
+      <x:c r="L26" s="44" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="M26" s="18" t="str">
+        <x:v>codex/moves-ai-liability-retrofit: labels Moves deliverables as AI Draft and keeps edit-before-commit / human-review language visible.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -7825,15 +7817,11 @@
           <x:t xml:space="preserve">Anytime</x:t>
         </x:is>
       </x:c>
-      <x:c r="L27" s="44" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M27" s="18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
+      <x:c r="L27" s="44" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="M27" s="18" t="str">
+        <x:v>codex/moves-ai-liability-retrofit: requires explicit human rationale before phase advance through API and agent tool paths.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">

</xml_diff>

<commit_message>
fix(moves): finish AI liability tracker controls
</commit_message>
<xml_diff>
--- a/docs/planning/ABARVA_PILOT_READINESS_PLAN.xlsx
+++ b/docs/planning/ABARVA_PILOT_READINESS_PLAN.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R2fa155bca9184c28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Ra751f8589b5f4dc3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan" sheetId="3" r:id="R2ba836e4f62f4681"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Queue" sheetId="4" r:id="Rcd96f3fadf154750"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance" sheetId="5" r:id="Re2f9f7c512b6412f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pricing" sheetId="6" r:id="R3a9496baee504c9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost Model" sheetId="7" r:id="R003202e93e884977"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BC - PHS" sheetId="8" r:id="Rb50ecf56ccf74679"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BC - Surekha" sheetId="9" r:id="R3fda1d3bdfe44112"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BC - Delta" sheetId="10" r:id="R9a8442473fe54da2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Pack" sheetId="11" r:id="R1a189b3f5ce14818"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Redline Brief" sheetId="12" r:id="R3152d3b9b0544921"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="13" r:id="R1437e39d35404035"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R3d57cad102034769"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R8855b95884884deb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan" sheetId="3" r:id="R034fe3b4b4ac4250"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Queue" sheetId="4" r:id="R431e77f3eb444928"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance" sheetId="5" r:id="Rca9d0af36e4f4abb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pricing" sheetId="6" r:id="R75e9fec23e2043e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost Model" sheetId="7" r:id="Raf72b385cbb8409b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BC - PHS" sheetId="8" r:id="R2acda9297e154320"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BC - Surekha" sheetId="9" r:id="R766ba48c37074475"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BC - Delta" sheetId="10" r:id="R1e5bff3a0dbf462f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Pack" sheetId="11" r:id="R44f3b0d805c640f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Redline Brief" sheetId="12" r:id="Rcbc3f432df8246bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="13" r:id="R058fc7ca8f504a28"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4567,7 +4567,7 @@
       </x:c>
       <x:c r="C7" s="7" t="n">
         <x:f>COUNTIF(Plan!L5:L333,"Done")</x:f>
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G7" s="6" t="inlineStr">
         <x:is>
@@ -4599,7 +4599,7 @@
       </x:c>
       <x:c r="C8" s="7" t="n">
         <x:f>COUNTIF(Plan!L5:L333,"In progress")</x:f>
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G8" s="6" t="inlineStr">
         <x:is>
@@ -4695,7 +4695,7 @@
       </x:c>
       <x:c r="C11" s="11" t="n">
         <x:f>IFERROR(C7/C6,0)</x:f>
-        <x:v>0.00303951367781155</x:v>
+        <x:v>0.0121580547112462</x:v>
       </x:c>
       <x:c r="G11" s="6" t="inlineStr">
         <x:is>
@@ -4845,11 +4845,11 @@
       </x:c>
       <x:c r="D15" s="9" t="n">
         <x:f>COUNTIFS(Plan!E5:E333,"P0",Plan!L5:L333,"Done")</x:f>
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E15" s="10" t="n">
         <x:f>IFERROR(D15/C15,0)</x:f>
-        <x:v>0.004629629629629629</x:v>
+        <x:v>0.018518518518518517</x:v>
       </x:c>
       <x:c r="G15" s="6" t="inlineStr">
         <x:is>
@@ -4883,7 +4883,7 @@
       </x:c>
       <x:c r="O15" s="9" t="n">
         <x:f>COUNTIFS(Plan!K5:K333,"Pre-Resign",Plan!L5:L333,"Done")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -5042,7 +5042,7 @@
       </x:c>
       <x:c r="O18" s="9" t="n">
         <x:f>COUNTIFS(Plan!K5:K333,"Anytime",Plan!L5:L333,"Done")</x:f>
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -5086,15 +5086,15 @@
       </x:c>
       <x:c r="I20" s="9" t="n">
         <x:f>COUNTIFS(Plan!B5:B333,"AI Liability Defense",Plan!L5:L333,"Done")</x:f>
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J20" s="9" t="n">
         <x:f>COUNTIFS(Plan!B5:B333,"AI Liability Defense",Plan!L5:L333,"In progress")</x:f>
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K20" s="10" t="n">
         <x:f>IFERROR(I20/H20,0)</x:f>
-        <x:v>0.02040816326530612</x:v>
+        <x:v>0.08163265306122448</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -5178,11 +5178,11 @@
       </x:c>
       <x:c r="D23" s="9" t="n">
         <x:f>COUNTIFS(Plan!F5:F333,"2. CLAUDE DOES IT",Plan!L5:L333,"Done")</x:f>
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E23" s="10" t="n">
         <x:f>IFERROR(D23/C23,0)</x:f>
-        <x:v>0.005291005291005291</x:v>
+        <x:v>0.021164021164021163</x:v>
       </x:c>
       <x:c r="F23" s="36" t="n"/>
       <x:c r="G23" s="36" t="n"/>
@@ -7692,10 +7692,10 @@
         </x:is>
       </x:c>
       <x:c r="L25" s="44" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M25" s="18" t="str">
-        <x:v>codex/moves-ai-liability-retrofit: adds 20-char human gate rationale and shared AI decision evidence packet to Moves phase-gate approval paths.</x:v>
+        <x:v>Implemented in codex/moves-ai-liability-retrofit: gate approvals require a human justification and create shared AI decision evidence bundles/audit references.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -7755,10 +7755,10 @@
         </x:is>
       </x:c>
       <x:c r="L26" s="44" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M26" s="18" t="str">
-        <x:v>codex/moves-ai-liability-retrofit: labels Moves deliverables as AI Draft and keeps edit-before-commit / human-review language visible.</x:v>
+        <x:v>Implemented in codex/moves-ai-liability-retrofit: Moves deliverables carry AI Draft labels plus edit-before-commit human-review requirements in the view model and UI.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -7818,10 +7818,10 @@
         </x:is>
       </x:c>
       <x:c r="L27" s="44" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M27" s="18" t="str">
-        <x:v>codex/moves-ai-liability-retrofit: requires explicit human rationale before phase advance through API and agent tool paths.</x:v>
+        <x:v>Implemented in codex/moves-ai-liability-retrofit: phase advance API, UI, and Nexus tool require explicit human rationale before commit.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">

</xml_diff>

<commit_message>
docs(governance): add AI liability catalogs
</commit_message>
<xml_diff>
--- a/docs/planning/ABARVA_PILOT_READINESS_PLAN.xlsx
+++ b/docs/planning/ABARVA_PILOT_READINESS_PLAN.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R3d57cad102034769"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R8855b95884884deb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan" sheetId="3" r:id="R034fe3b4b4ac4250"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Queue" sheetId="4" r:id="R431e77f3eb444928"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance" sheetId="5" r:id="Rca9d0af36e4f4abb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pricing" sheetId="6" r:id="R75e9fec23e2043e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost Model" sheetId="7" r:id="Raf72b385cbb8409b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BC - PHS" sheetId="8" r:id="R2acda9297e154320"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BC - Surekha" sheetId="9" r:id="R766ba48c37074475"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BC - Delta" sheetId="10" r:id="R1e5bff3a0dbf462f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Pack" sheetId="11" r:id="R44f3b0d805c640f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Redline Brief" sheetId="12" r:id="Rcbc3f432df8246bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="13" r:id="R058fc7ca8f504a28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R79630c3435ff48bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R35c24e02d0fb4c50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan" sheetId="3" r:id="R3495243f5a32494e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Queue" sheetId="4" r:id="R2618c3e7635b41af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance" sheetId="5" r:id="R6936f795e17540fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pricing" sheetId="6" r:id="Re88db63e07b94b05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost Model" sheetId="7" r:id="Rd27a19a2d1dd4567"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BC - PHS" sheetId="8" r:id="R6fe27779c7e746dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BC - Surekha" sheetId="9" r:id="R6715b825d1534983"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BC - Delta" sheetId="10" r:id="R7b5c4ac4499046f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Pack" sheetId="11" r:id="Rfd06cfd456ff4524"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Redline Brief" sheetId="12" r:id="R02402d639c49408d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="13" r:id="Rbffdf680160648e3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4567,7 +4567,7 @@
       </x:c>
       <x:c r="C7" s="7" t="n">
         <x:f>COUNTIF(Plan!L5:L333,"Done")</x:f>
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G7" s="6" t="inlineStr">
         <x:is>
@@ -4663,7 +4663,7 @@
       </x:c>
       <x:c r="C10" s="7" t="n">
         <x:f>COUNTIF(Plan!L5:L333,"Not started")</x:f>
-        <x:v>325</x:v>
+        <x:v>323</x:v>
       </x:c>
       <x:c r="G10" s="6" t="inlineStr">
         <x:is>
@@ -4695,7 +4695,7 @@
       </x:c>
       <x:c r="C11" s="11" t="n">
         <x:f>IFERROR(C7/C6,0)</x:f>
-        <x:v>0.0121580547112462</x:v>
+        <x:v>0.0182370820668693</x:v>
       </x:c>
       <x:c r="G11" s="6" t="inlineStr">
         <x:is>
@@ -4845,11 +4845,11 @@
       </x:c>
       <x:c r="D15" s="9" t="n">
         <x:f>COUNTIFS(Plan!E5:E333,"P0",Plan!L5:L333,"Done")</x:f>
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E15" s="10" t="n">
         <x:f>IFERROR(D15/C15,0)</x:f>
-        <x:v>0.018518518518518517</x:v>
+        <x:v>0.027777777777777776</x:v>
       </x:c>
       <x:c r="G15" s="6" t="inlineStr">
         <x:is>
@@ -5042,7 +5042,7 @@
       </x:c>
       <x:c r="O18" s="9" t="n">
         <x:f>COUNTIFS(Plan!K5:K333,"Anytime",Plan!L5:L333,"Done")</x:f>
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -5086,7 +5086,7 @@
       </x:c>
       <x:c r="I20" s="9" t="n">
         <x:f>COUNTIFS(Plan!B5:B333,"AI Liability Defense",Plan!L5:L333,"Done")</x:f>
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="J20" s="9" t="n">
         <x:f>COUNTIFS(Plan!B5:B333,"AI Liability Defense",Plan!L5:L333,"In progress")</x:f>
@@ -5094,7 +5094,7 @@
       </x:c>
       <x:c r="K20" s="10" t="n">
         <x:f>IFERROR(I20/H20,0)</x:f>
-        <x:v>0.08163265306122448</x:v>
+        <x:v>0.12244897959183673</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -5178,11 +5178,11 @@
       </x:c>
       <x:c r="D23" s="9" t="n">
         <x:f>COUNTIFS(Plan!F5:F333,"2. CLAUDE DOES IT",Plan!L5:L333,"Done")</x:f>
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E23" s="10" t="n">
         <x:f>IFERROR(D23/C23,0)</x:f>
-        <x:v>0.021164021164021163</x:v>
+        <x:v>0.031746031746031744</x:v>
       </x:c>
       <x:c r="F23" s="36" t="n"/>
       <x:c r="G23" s="36" t="n"/>
@@ -7423,15 +7423,11 @@
           <x:t xml:space="preserve">Anytime</x:t>
         </x:is>
       </x:c>
-      <x:c r="L21" s="44" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M21" s="18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
+      <x:c r="L21" s="44" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="M21" s="18" t="str">
+        <x:v>PR #2723: docs/legal/AI_CONSEQUENTIAL_ACTION_CATALOG.md catalogs verified cross-module consequential actions.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -7490,15 +7486,11 @@
           <x:t xml:space="preserve">Anytime</x:t>
         </x:is>
       </x:c>
-      <x:c r="L22" s="44" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M22" s="18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
+      <x:c r="L22" s="44" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="M22" s="18" t="str">
+        <x:v>PR #2723: docs/legal/AI_GENERATED_UI_CATALOG.md catalogs verified generated-output UI surfaces.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">

</xml_diff>

<commit_message>
Document Supabase retirement readiness blockers
Co-authored-by: anandsundaram-hash <anandsundaram-hash@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/planning/ABARVA_PILOT_READINESS_PLAN.xlsx
+++ b/docs/planning/ABARVA_PILOT_READINESS_PLAN.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R79630c3435ff48bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R35c24e02d0fb4c50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan" sheetId="3" r:id="R3495243f5a32494e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Queue" sheetId="4" r:id="R2618c3e7635b41af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance" sheetId="5" r:id="R6936f795e17540fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pricing" sheetId="6" r:id="Re88db63e07b94b05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost Model" sheetId="7" r:id="Rd27a19a2d1dd4567"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BC - PHS" sheetId="8" r:id="R6fe27779c7e746dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BC - Surekha" sheetId="9" r:id="R6715b825d1534983"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BC - Delta" sheetId="10" r:id="R7b5c4ac4499046f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Pack" sheetId="11" r:id="Rfd06cfd456ff4524"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Redline Brief" sheetId="12" r:id="R02402d639c49408d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="13" r:id="Rbffdf680160648e3"/>
-  </x:sheets>
-</x:workbook>
+<ns0:workbook xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <ns0:sheets>
+    <ns0:sheet name="README" sheetId="1" r:id="R79630c3435ff48bb"/>
+    <ns0:sheet name="Dashboard" sheetId="2" r:id="R35c24e02d0fb4c50"/>
+    <ns0:sheet name="Plan" sheetId="3" r:id="R3495243f5a32494e"/>
+    <ns0:sheet name="Codex Queue" sheetId="4" r:id="R2618c3e7635b41af"/>
+    <ns0:sheet name="Governance" sheetId="5" r:id="R6936f795e17540fa"/>
+    <ns0:sheet name="Pricing" sheetId="6" r:id="Re88db63e07b94b05"/>
+    <ns0:sheet name="Cost Model" sheetId="7" r:id="Rd27a19a2d1dd4567"/>
+    <ns0:sheet name="BC - PHS" sheetId="8" r:id="R6fe27779c7e746dd"/>
+    <ns0:sheet name="BC - Surekha" sheetId="9" r:id="R6715b825d1534983"/>
+    <ns0:sheet name="BC - Delta" sheetId="10" r:id="R7b5c4ac4499046f5"/>
+    <ns0:sheet name="Security Pack" sheetId="11" r:id="Rfd06cfd456ff4524"/>
+    <ns0:sheet name="Redline Brief" sheetId="12" r:id="R02402d639c49408d"/>
+    <ns0:sheet name="Risks" sheetId="13" r:id="Rbffdf680160648e3"/>
+    <ns0:sheet name="Legacy Shutdown" sheetId="14" r:id="rIdLegacyShutdown6783"/>
+  </ns0:sheets>
+</ns0:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4477,6 +4478,87 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <ns0:dimension ref="A1:F2"/>
+  <ns0:sheetFormatPr defaultRowHeight="15"/>
+  <ns0:sheetData>
+    <ns0:row r="1">
+      <ns0:c r="A1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Component</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Status</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Gate Summary</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Evidence</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Next Action</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Updated UTC</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="2">
+      <ns0:c r="A2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Supabase</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>BLOCKED</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Runtime Azure-only; data parity, backup/restore, signed-in QA, and final approval gates are not all green.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>docs/build/legacy-shutdown-readiness/README.md</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Run source-backed reconciliation for all required tables, migrate missing rows if any, complete backup/restore and QA, then ask Anand for approval only after a green report.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2026-06-07T15:53:36Z</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+  </ns0:sheetData>
+  <ns0:cols>
+    <ns0:col min="1" max="1" width="18" customWidth="1"/>
+    <ns0:col min="2" max="2" width="18" customWidth="1"/>
+    <ns0:col min="3" max="3" width="72" customWidth="1"/>
+    <ns0:col min="4" max="4" width="52" customWidth="1"/>
+    <ns0:col min="5" max="5" width="96" customWidth="1"/>
+    <ns0:col min="6" max="6" width="24" customWidth="1"/>
+  </ns0:cols>
+</ns0:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>

</xml_diff>